<commit_message>
correzione layout ottimizzazione spazi codici errori
</commit_message>
<xml_diff>
--- a/errori-en.xlsx
+++ b/errori-en.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\f.refrigeri\Documents\Documenti Flavio\MicroserviziWeb\micro-tools-suite\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{528FC8DD-74F4-4AB0-9751-940FCC027B6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{499579FC-B721-4BD1-8ED5-C2BB2E773361}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32160" yWindow="4740" windowWidth="21600" windowHeight="11292" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="95">
   <si>
     <t>Brand</t>
   </si>
@@ -198,31 +198,6 @@
 Single or double basket: Single basket
 Connectivity: No connection
 Dishwasher-safe components: Yes</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> "E1"
-The air fryer may have been stored in a place that was too cold.
-If the device has been stored in a low-temperature environment,
-let it warm up to room temperature for at least 15 minutes before plugging it back in.
-If the problem persists, call the Philips telephone support service
-or go to the customer service center in your country.
-The air fryer display shows the codes
-"E4"
-The device shows an error. Unplug the device and plug it back in.
-If the problem persists, call the Philips telephone support service
-or go to the customer service center in your country.
-"E6"
-The device shows an error. Unplug the device and plug it back in.
-If the problem persists, call the Philips telephone support service
-or go to the customer service center in your country.
- "E9"
-The device shows an error. Unplug the device and plug it back in.
-If the problem persists, call the Philips telephone support service
-or go to the customer service center in your country.
-"E12"
-The device shows an error. Unplug the device and plug it back in.
-If the problem persists, call the Philips telephone support service
-or go to the customer service center in your country.</t>
   </si>
   <si>
     <t>https://www.home.id/it-IT/NA221</t>
@@ -1163,6 +1138,170 @@
 Turn off and unplug the air fryer and let it cool down completely.
 If the display still shows "E28", contact Customer Service (see page 25).</t>
   </si>
+  <si>
+    <t>MAF-D1001</t>
+  </si>
+  <si>
+    <t>Xiaomi MAF-D1001 Smart Double Stack Air Fryer User Manual - Manuals+</t>
+  </si>
+  <si>
+    <t>MAF-W6051</t>
+  </si>
+  <si>
+    <t>Troubleshooting - Xiaomi Smart Air Fryer 6,5 User Manual [Page 10] | ManualsLib</t>
+  </si>
+  <si>
+    <t>Name
+Xiaomi Dual Zone Air Fryer 10L
+Model
+MAF-D1001
+Color
+Black
+Rated power
+2700 W (1150 W left + 1450 W right)
+Rated voltage
+220-240 V~
+Rated frequency
+50-60 Hz
+Rated capacity
+10 L (3.5 L left + 6.5 L right)</t>
+  </si>
+  <si>
+    <t>English
+Product name
+Xiaomi Air Fryer 6.5L
+Product model
+MAF-W6051
+Product color
+White
+Black
+Rated power
+1700 W
+Rated voltage
+220-240 V~
+Rated frequency
+50-60 Hz
+Rated capacity
+6.5 L</t>
+  </si>
+  <si>
+    <t>Xiaomi</t>
+  </si>
+  <si>
+    <t>Xiaomi Dual Zone Air Fryer 10L</t>
+  </si>
+  <si>
+    <t>Xiaomi Air Fryer 6,5L</t>
+  </si>
+  <si>
+    <t>English
+"The air fryer doesn't function."
+Classification: Power / Assembly Check
+Severity: Low
+"E1"
+Classification: Hardware Repair
+Severity: High
+"E2"
+Classification: Hardware Repair
+Severity: High
+"The fan doesn't rotate."
+Classification: Hardware Repair
+Severity: High
+"White smoke is coming out."
+Classification: Cleaning / Normal Operation
+Severity: Low
+"Can't insert the basket into the air fryer smoothly."
+Classification: Usage / Capacity Error
+Severity: Low
+"The schedule function doesn't function as requested."
+Classification: Software / Setup Error
+Severity: Low
+"Wi-Fi can't be connected."
+Classification: Network / App Error
+Severity: Low
+"Unable to connect the air fryer."
+Classification: Network / App Error
+Severity: Low</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"The air fryer doesn't function."
+Classification: Power / Assembly Check
+Severity: Low  
+"E1"
+Classification: Hardware Repair
+Severity: High   
+"E2"
+Classification: Hardware Repair
+Severity: High   
+"The fan doesn't rotate."
+Classification: Hardware Repair
+Severity: High   
+"White smoke is coming out."
+Classification: Cleaning / Normal Operation
+Severity: Low  
+"Can't insert the basket into the air fryer smoothly."
+Classification: Usage / Capacity Error
+Severity: Low  </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> "E1"
+The air fryer may have been stored in a place that was too cold.
+If the device has been stored in a low-temperature environment,
+let it warm up to room temperature for at least 15 minutes before plugging it back in.
+If the problem persists, call the Philips telephone support service
+or go to the customer service center in your country.
+The air fryer the codes
+"E4"
+The device shows an error. Unplug the device and plug it back in.
+If the problem persists, call the Philips telephone support service
+or go to the customer service center in your country.
+"E6"
+The device shows an error. Unplug the device and plug it back in.
+If the problem persists, call the Philips telephone support service
+or go to the customer service center in your country.
+ "E9"
+The device shows an error. Unplug the device and plug it back in.
+If the problem persists, call the Philips telephone support service
+or go to the customer service center in your country.
+"E12"
+The device shows an error. Unplug the device and plug it back in.
+If the problem persists, call the Philips telephone support service
+or go to the customer service center in your country.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"The air fryer doesn't function."
+The air fryer is not connected to a power supply; plug the power cord into a grounded electrical outlet. The basket is not pushed into place; pull out the basket and push it back into place.   
+"E1"
+The sensor has a broken circuit; contact the after-sales service team.   
+"E2"
+The sensor has a short circuit; contact the after-sales service team.  
+ "The fan doesn't rotate."
+The fan blade is stuck; contact the after-sales service team. The motor is damaged or other components have a broken circuit; contact the after-sales service team.   
+"White smoke is coming out."
+Cooking oily ingredients: when you fry ingredients containing more fat, there will be a lot of smoke, which is normal. The air fryer still contains grease residue from the previous cooking program; ensure that you clean the air fryer after each cooking program.   
+"Can't insert the basket into the air fryer smoothly."
+Too many ingredients in the basket; the ingredients in the basket can't exceed the maximum mark. The basket is not properly inserted; properly insert the basket. </t>
+  </si>
+  <si>
+    <t>"The air fryer doesn't function."
+The air fryer is not connected to a power supply; plug the power cord into a grounded electrical outlet. The basket is not pushed into place; pull out the basket and push it back into place.
+"E1"
+The sensor has a broken circuit; contact the after-sales service team.
+"E2"
+The sensor has a short circuit; contact the after-sales service team.
+"The fan doesn't rotate."
+The fan blade is stuck; contact the after-sales service team. The motor is damaged or other components have a broken circuit; contact the after-sales service team.
+"White smoke is coming out."
+Cooking oily ingredients: when you fry ingredients containing more fat, there will be a lot of smoke, which is normal. The air fryer still contains grease residue from the previous cooking program; ensure that you clean the air fryer after each cooking program.
+"Can't insert the basket into the air fryer smoothly."
+Too many ingredients in the basket; the ingredients in the basket can't exceed the maximum mark. The basket is not properly inserted; properly insert the basket.   
+"The schedule function doesn't function as requested."
+The scheduled time is too short; the scheduled time should be longer than the cooking time. The scheduled time is not saved; the scheduled time should be saved and carried out by pressing the control knob.   
+"Wi-Fi can't be connected."
+The Mi Home/Xiaomi Home app is not the latest version; update the Mi Home/Xiaomi Home app to the latest version. The Wi-Fi signal is weak; move to a location where the signal is strong enough.   
+"Unable to connect the air fryer."
+Wi-Fi cannot be connected; check whether the Wi-Fi is connected normally or reset the Wi-Fi to reconnect.</t>
+  </si>
 </sst>
 </file>
 
@@ -1214,7 +1353,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1237,6 +1376,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Collegamento ipertestuale" xfId="1" builtinId="8"/>
@@ -1572,7 +1712,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="2" customWidth="1"/>
@@ -1609,7 +1749,7 @@
         <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1638,7 +1778,7 @@
         <v>14</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1655,19 +1795,19 @@
         <v>17</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>18</v>
+        <v>92</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1675,28 +1815,28 @@
         <v>8</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>23</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1704,271 +1844,319 @@
         <v>8</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="F5" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="G5" s="6" t="s">
-        <v>30</v>
-      </c>
       <c r="H5" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="180" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="C6" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="D6" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="E6" s="5" t="s">
         <v>34</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>35</v>
       </c>
       <c r="F6" s="4"/>
       <c r="G6" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="285" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D7" s="1" t="s">
-        <v>39</v>
-      </c>
       <c r="E7" s="7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F7" s="5"/>
       <c r="G7" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="315" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="E8" s="5" t="s">
         <v>43</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>44</v>
       </c>
       <c r="F8" s="5"/>
       <c r="G8" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="210" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B9" t="s">
+        <v>45</v>
+      </c>
+      <c r="C9" t="s">
         <v>46</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>47</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" s="1" t="s">
         <v>48</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>49</v>
       </c>
       <c r="F9" s="1"/>
       <c r="G9" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="270" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B10" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C10" t="s">
-        <v>47</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>52</v>
-      </c>
       <c r="E10" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F10" s="1"/>
       <c r="G10" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B11" t="s">
+        <v>52</v>
+      </c>
+      <c r="C11" t="s">
         <v>53</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D11" s="1" t="s">
-        <v>55</v>
-      </c>
       <c r="E11" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F11" s="1"/>
       <c r="G11" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="270" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C12" t="s">
         <v>57</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="E12" s="1" t="s">
         <v>59</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>60</v>
       </c>
       <c r="F12" s="1"/>
       <c r="G12" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C13" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D13" s="1" t="s">
-        <v>59</v>
-      </c>
       <c r="E13" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F13" s="1"/>
       <c r="G13" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="180" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B14" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C14" t="s">
         <v>63</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>64</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" s="1" t="s">
         <v>65</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>66</v>
       </c>
       <c r="F14" s="1"/>
       <c r="G14" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="345" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C15" t="s">
+        <v>81</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="F15" s="2"/>
+      <c r="G15" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C16" t="s">
+        <v>83</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="F16" s="2"/>
+      <c r="G16" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -1979,8 +2167,10 @@
     <hyperlink ref="H5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
     <hyperlink ref="B13" r:id="rId5" display="https://cosori.com/collections/air-fryers/products/cosori-9-0-quart-dual-basket-air-fryer" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
     <hyperlink ref="B14" r:id="rId6" display="https://cosori.com/collections/air-fryers/products/pro-le-5-0-quart-air-fryer" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="G15" r:id="rId7" display="https://it.manuals.plus/xiaomi/maf-d1001-smart-double-stack-air-fryer-manual" xr:uid="{E64C8336-3816-4B51-852A-D3A7089CDCD4}"/>
+    <hyperlink ref="G16" r:id="rId8" display="https://www.manualslib.com/manual/3272450/Xiaomi-Smart-Air-Fryer-6-5.html?page=10" xr:uid="{BFFA95BB-C18A-4B00-B580-7E7CF29DC0AB}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId9"/>
 </worksheet>
 </file>
</xml_diff>